<commit_message>
Changes to body of email property in JSON payload to be inserted into DB for orders-stuck-in-created-15-mins
</commit_message>
<xml_diff>
--- a/stuck-in-created-15-minutes/WarehouseDetail_records(stuck-in-created-15-minutes).xlsx
+++ b/stuck-in-created-15-minutes/WarehouseDetail_records(stuck-in-created-15-minutes).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rndc/Desktop/Work related/Documents/stuck-in-created-15-minutes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB92D367-C437-224C-B0D5-8522D9CEC74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE137E7-26A8-DC41-9D09-AD41CC98C109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
   </bookViews>
@@ -1514,7 +1514,7 @@
     <t>TBD</t>
   </si>
   <si>
-    <t>{"alertName":"ORDERS STUCK IN CREATED STATUS &gt; 15 MINUTES","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;&lt;br /&gt;The alert condition for ''$name$'' was triggered.&lt;br /&gt;&lt;br /&gt;***MSP TO CLEAN UP***&lt;br /&gt;&lt;br /&gt;Note: Manhattan Case 8199748 is created.&lt;br /&gt;&lt;br /&gt;Description: &lt;br /&gt;1. Go to System Management&gt;Tranlog Summary&gt;XNT_DCO_OriginalOrders &lt;br /&gt;2. Type in the Order Number for the Order Stuck in Created Status&lt;br /&gt;3. Pull the JSON for the order and Put it in this API, but do not run Yet&lt;br /&gt;            {{app_host}}/dcorder/api/dcorder/originalOrder/save&lt;br /&gt;4. Delete the Original Order Using this API, Replace XXX with the House, and update the Order_Id&lt;br /&gt;            {{app_host}}/dcorder/api/dcorder/originalOrder/bulkDelete&lt;br /&gt;                {&lt;br /&gt;    'Data': [&lt;br /&gt;        {&lt;br /&gt;            'OrderId': '123123',&lt;br /&gt;            'OriginFacilityId': 'XXX'&lt;br /&gt;        }&lt;br /&gt;    ]&lt;br /&gt;}&lt;br /&gt;5. Delete the Order Using this API, Replace XXX with the House, and update the Order_Id&lt;br /&gt;                {{app_host}}/dcorder/api/dcorder/order/bulkDelete&lt;br /&gt;                {&lt;br /&gt;    'Data': [&lt;br /&gt;        {&lt;br /&gt;            'OriginalOrderId': '123123',&lt;br /&gt;            'OriginFacilityId': 'XXX'&lt;br /&gt;        }&lt;br /&gt;    ]&lt;br /&gt;}&lt;br /&gt;6. Reimport the Order using the JSON from Step 3&lt;br /&gt;&lt;/body&gt;&lt;br /&gt;&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"wmsinternal@RNDC-USA.COM, WMSConsultant@rndc-usa.com, Mcurtis@manh.com, WMSMSPSupport@RNDC-USA.COM,DL_MANH_RNDC_MAWM_PSO@manh.com,DL_RNDC_MAWM_CSO@manh.com","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT OO.ORG_ID 'Org ID', OO.CREATED_TIMESTAMP 'Created Timestamp',OO.BILLING_ACCOUNT_NUMBER 'Billing Acct #', OO.ORIGINAL_ORDER_ID 'Original Order ID', OO.ORDER_TYPE 'Order Type', OO.MAXIMUM_STATUS 'Maximum Status', STATUS.DESCRIPTION 'Description', OO.CANCELLED 'Cancelled', OO.BILL_TO_NAME 'Bill-to Name', OO.EXT_ROUTE_ID 'Ext Route ID', OO.EXT_SHIPMENT_STOP_NUMBER 'Ext Shipment Stop #' FROM default_dcorder.DCO_ORIGINAL_ORDER OO JOIN default_dcorder.DCO_ORDER_STATUS STATUS ON OO.MAXIMUM_STATUS = STATUS.ORDER_STATUS_ID WHERE 1=1 AND (OO.MAXIMUM_STATUS = '0000' or OO.MAXIMUM_STATUS = '0000') AND OO.CREATED_TIMESTAMP &lt;= DATE_SUB(now(), INTERVAL '10' MINUTE);"}'</t>
+    <t>{"alertName":"ORDERS STUCK IN CREATED STATUS &gt; 15 MINUTES","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;&lt;br /&gt;The alert condition for ''$name$'' was triggered.&lt;br /&gt;&lt;br /&gt;***MSP TO CLEAN UP***&lt;br /&gt;&lt;br /&gt;Note: Manhattan Case 8199748 is created.&lt;br /&gt;&lt;br /&gt;Description: &lt;br /&gt;1. Go to System Management&gt;Tranlog Summary&gt;XNT_DCO_OriginalOrders &lt;br /&gt;2. Type in the Order Number for the Order Stuck in Created Status&lt;br /&gt;3. Pull the JSON for the order and Put it in this API, but do not run Yet&lt;br /&gt;            {{app_host}}/dcorder/api/dcorder/originalOrder/save&lt;br /&gt;4. Delete the Original Order Using this API, Replace XXX with the House, and update the Order_Id&lt;br /&gt;            {{app_host}}/dcorder/api/dcorder/originalOrder/bulkDelete&lt;br /&gt;                {&lt;br /&gt;    ''Data'': [&lt;br /&gt;        {&lt;br /&gt;            ''OrderId'': ''123123'',&lt;br /&gt;            ''OriginFacilityId'': ''XXX''&lt;br /&gt;        }&lt;br /&gt;    ]&lt;br /&gt;}&lt;br /&gt;5. Delete the Order Using this API, Replace XXX with the House, and update the Order_Id&lt;br /&gt;                {{app_host}}/dcorder/api/dcorder/order/bulkDelete&lt;br /&gt;                {&lt;br /&gt;    ''Data'': [&lt;br /&gt;        {&lt;br /&gt;            ''OriginalOrderId'': ''123123'',&lt;br /&gt;            ''OriginFacilityId'': ''XXX''&lt;br /&gt;        }&lt;br /&gt;    ]&lt;br /&gt;}&lt;br /&gt;6. Reimport the Order using the JSON from Step 3&lt;br /&gt;&lt;/body&gt;&lt;br /&gt;&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"wmsinternal@RNDC-USA.COM, WMSConsultant@rndc-usa.com, Mcurtis@manh.com, WMSMSPSupport@RNDC-USA.COM,DL_MANH_RNDC_MAWM_PSO@manh.com,DL_RNDC_MAWM_CSO@manh.com","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT OO.ORG_ID 'Org ID', OO.CREATED_TIMESTAMP 'Created Timestamp',OO.BILLING_ACCOUNT_NUMBER 'Billing Acct #', OO.ORIGINAL_ORDER_ID 'Original Order ID', OO.ORDER_TYPE 'Order Type', OO.MAXIMUM_STATUS 'Maximum Status', STATUS.DESCRIPTION 'Description', OO.CANCELLED 'Cancelled', OO.BILL_TO_NAME 'Bill-to Name', OO.EXT_ROUTE_ID 'Ext Route ID', OO.EXT_SHIPMENT_STOP_NUMBER 'Ext Shipment Stop #' FROM default_dcorder.DCO_ORIGINAL_ORDER OO JOIN default_dcorder.DCO_ORDER_STATUS STATUS ON OO.MAXIMUM_STATUS = STATUS.ORDER_STATUS_ID WHERE 1=1 AND (OO.MAXIMUM_STATUS = '0000' or OO.MAXIMUM_STATUS = '0000') AND OO.CREATED_TIMESTAMP &lt;= DATE_SUB(now(), INTERVAL '10' MINUTE);"}'</t>
   </si>
 </sst>
 </file>

</xml_diff>